<commit_message>
add data of day two of experiment
</commit_message>
<xml_diff>
--- a/data/raw/p_12.09.26_cupins.xlsx
+++ b/data/raw/p_12.09.26_cupins.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cmilacristina/ecopan/fase3/cupins_ecopan/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{652342C9-BFDA-3040-8C43-401F552EE078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2083592-62B9-8840-83F8-A04A42B6ABD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{04C7B980-90C4-4B4B-BE90-0937D8BBCD2B}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="27">
   <si>
     <t>ninho</t>
   </si>
@@ -61,6 +61,9 @@
     <t>c3</t>
   </si>
   <si>
+    <t>c4</t>
+  </si>
+  <si>
     <t>c7</t>
   </si>
   <si>
@@ -104,6 +107,9 @@
   </si>
   <si>
     <t>volume</t>
+  </si>
+  <si>
+    <t>c2</t>
   </si>
   <si>
     <t>t_recrut</t>
@@ -530,33 +536,33 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>3</v>
@@ -565,30 +571,57 @@
         <f>D2-C2</f>
         <v>0</v>
       </c>
+      <c r="G2" s="3">
+        <v>11</v>
+      </c>
+      <c r="H2" s="3">
+        <v>21</v>
+      </c>
+      <c r="I2" s="3">
+        <v>13</v>
+      </c>
       <c r="J2" s="4">
         <f>I2*H2*G2*(4/3)*(3.14159)/1000</f>
-        <v>0</v>
+        <v>12.578926359999999</v>
       </c>
     </row>
     <row r="3" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="C3" s="2">
+        <v>0</v>
+      </c>
+      <c r="D3" s="2">
+        <v>172</v>
+      </c>
       <c r="E3" s="2">
-        <f t="shared" ref="E3:E37" si="0">D3-C3</f>
-        <v>0</v>
+        <f t="shared" ref="E3:E43" si="0">D3-C3</f>
+        <v>172</v>
+      </c>
+      <c r="F3" s="2">
+        <v>27</v>
+      </c>
+      <c r="G3" s="2">
+        <v>11</v>
+      </c>
+      <c r="H3" s="2">
+        <v>21</v>
+      </c>
+      <c r="I3" s="2">
+        <v>13</v>
       </c>
       <c r="J3" s="5">
         <f>I3*H3*G3*(4/3)*(3.14159)/1000</f>
-        <v>0</v>
+        <v>12.578926359999999</v>
       </c>
     </row>
     <row r="4" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>5</v>
@@ -622,7 +655,7 @@
     </row>
     <row r="5" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>3</v>
@@ -631,14 +664,23 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="G5" s="3">
+        <v>10</v>
+      </c>
+      <c r="H5" s="3">
+        <v>20</v>
+      </c>
+      <c r="I5" s="3">
+        <v>12</v>
+      </c>
       <c r="J5" s="4">
-        <f t="shared" ref="J5:J37" si="1">I5*H5*G5*(4/3)*(3.14159)/1000</f>
-        <v>0</v>
+        <f t="shared" ref="J5:J43" si="1">I5*H5*G5*(4/3)*(3.14159)/1000</f>
+        <v>10.053087999999999</v>
       </c>
     </row>
     <row r="6" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>4</v>
@@ -647,24 +689,30 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="F6" s="2">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2">
+        <v>10</v>
+      </c>
+      <c r="H6" s="2">
+        <v>20</v>
+      </c>
+      <c r="I6" s="2">
+        <v>12</v>
+      </c>
       <c r="J6" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>10.053087999999999</v>
       </c>
     </row>
     <row r="7" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="2">
-        <v>0</v>
-      </c>
-      <c r="D7" s="2">
-        <v>0</v>
-      </c>
       <c r="E7" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -673,22 +721,22 @@
         <v>0</v>
       </c>
       <c r="G7" s="2">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H7" s="2">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="I7" s="2">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="J7" s="5">
         <f t="shared" si="1"/>
-        <v>22.988061226666666</v>
+        <v>10.053087999999999</v>
       </c>
     </row>
     <row r="8" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>3</v>
@@ -697,30 +745,57 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="G8" s="3">
+        <v>90</v>
+      </c>
+      <c r="H8" s="3">
+        <v>22</v>
+      </c>
+      <c r="I8" s="3">
+        <v>49</v>
+      </c>
       <c r="J8" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>406.39608240000001</v>
       </c>
     </row>
     <row r="9" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="C9" s="2">
+        <v>218</v>
+      </c>
+      <c r="D9" s="2">
+        <v>472</v>
+      </c>
       <c r="E9" s="2">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>254</v>
+      </c>
+      <c r="F9" s="2">
+        <v>3</v>
+      </c>
+      <c r="G9" s="2">
+        <v>90</v>
+      </c>
+      <c r="H9" s="2">
+        <v>22</v>
+      </c>
+      <c r="I9" s="2">
+        <v>49</v>
       </c>
       <c r="J9" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>406.39608240000001</v>
       </c>
     </row>
     <row r="10" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>5</v>
@@ -763,9 +838,18 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="G11" s="3">
+        <v>39</v>
+      </c>
+      <c r="H11" s="3">
+        <v>11</v>
+      </c>
+      <c r="I11" s="3">
+        <v>22</v>
+      </c>
       <c r="J11" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>39.533768559999999</v>
       </c>
     </row>
     <row r="12" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -775,13 +859,31 @@
       <c r="B12" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="C12" s="2">
+        <v>13</v>
+      </c>
+      <c r="D12" s="2">
+        <v>364</v>
+      </c>
       <c r="E12" s="2">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>351</v>
+      </c>
+      <c r="F12" s="2">
+        <v>5</v>
+      </c>
+      <c r="G12" s="2">
+        <v>39</v>
+      </c>
+      <c r="H12" s="2">
+        <v>11</v>
+      </c>
+      <c r="I12" s="2">
+        <v>22</v>
       </c>
       <c r="J12" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>39.533768559999999</v>
       </c>
     </row>
     <row r="13" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -829,9 +931,18 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="G14" s="3">
+        <v>46</v>
+      </c>
+      <c r="H14" s="3">
+        <v>27</v>
+      </c>
+      <c r="I14" s="3">
+        <v>22</v>
+      </c>
       <c r="J14" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>114.45440687999999</v>
       </c>
     </row>
     <row r="15" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -841,13 +952,31 @@
       <c r="B15" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="C15" s="2">
+        <v>9</v>
+      </c>
+      <c r="D15" s="2">
+        <v>336</v>
+      </c>
       <c r="E15" s="2">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>327</v>
+      </c>
+      <c r="F15" s="2">
+        <v>24</v>
+      </c>
+      <c r="G15" s="2">
+        <v>46</v>
+      </c>
+      <c r="H15" s="2">
+        <v>27</v>
+      </c>
+      <c r="I15" s="2">
+        <v>22</v>
       </c>
       <c r="J15" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>114.45440687999999</v>
       </c>
     </row>
     <row r="16" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -886,7 +1015,7 @@
     </row>
     <row r="17" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>3</v>
@@ -895,30 +1024,57 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="G17" s="3">
+        <v>26</v>
+      </c>
+      <c r="H17" s="3">
+        <v>19</v>
+      </c>
+      <c r="I17" s="3">
+        <v>23</v>
+      </c>
       <c r="J17" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>47.592994106666659</v>
       </c>
     </row>
     <row r="18" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="C18" s="2">
+        <v>0</v>
+      </c>
+      <c r="D18" s="2">
+        <v>480</v>
+      </c>
       <c r="E18" s="2">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>480</v>
+      </c>
+      <c r="F18" s="2">
+        <v>18</v>
+      </c>
+      <c r="G18" s="2">
+        <v>26</v>
+      </c>
+      <c r="H18" s="2">
+        <v>19</v>
+      </c>
+      <c r="I18" s="2">
+        <v>23</v>
       </c>
       <c r="J18" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>47.592994106666659</v>
       </c>
     </row>
     <row r="19" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>5</v>
@@ -952,7 +1108,7 @@
     </row>
     <row r="20" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>3</v>
@@ -961,30 +1117,57 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="G20" s="3">
+        <v>42</v>
+      </c>
+      <c r="H20" s="3">
+        <v>21</v>
+      </c>
+      <c r="I20" s="3">
+        <v>35</v>
+      </c>
       <c r="J20" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>129.30784439999999</v>
       </c>
     </row>
     <row r="21" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="C21" s="2">
+        <v>4</v>
+      </c>
+      <c r="D21" s="2">
+        <v>712</v>
+      </c>
       <c r="E21" s="2">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>708</v>
+      </c>
+      <c r="F21" s="2">
+        <v>29</v>
+      </c>
+      <c r="G21" s="2">
+        <v>42</v>
+      </c>
+      <c r="H21" s="2">
+        <v>21</v>
+      </c>
+      <c r="I21" s="2">
+        <v>35</v>
       </c>
       <c r="J21" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>129.30784439999999</v>
       </c>
     </row>
     <row r="22" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>5</v>
@@ -1018,7 +1201,7 @@
     </row>
     <row r="23" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>3</v>
@@ -1027,14 +1210,23 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="G23" s="3">
+        <v>44</v>
+      </c>
+      <c r="H23" s="3">
+        <v>24</v>
+      </c>
+      <c r="I23" s="3">
+        <v>33</v>
+      </c>
       <c r="J23" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>145.97083775999999</v>
       </c>
     </row>
     <row r="24" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>4</v>
@@ -1043,14 +1235,26 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="F24" s="2">
+        <v>0</v>
+      </c>
+      <c r="G24" s="2">
+        <v>44</v>
+      </c>
+      <c r="H24" s="2">
+        <v>24</v>
+      </c>
+      <c r="I24" s="2">
+        <v>33</v>
+      </c>
       <c r="J24" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>145.97083775999999</v>
       </c>
     </row>
     <row r="25" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>5</v>
@@ -1084,7 +1288,7 @@
     </row>
     <row r="26" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>3</v>
@@ -1093,30 +1297,57 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="G26" s="3">
+        <v>40</v>
+      </c>
+      <c r="H26" s="3">
+        <v>30</v>
+      </c>
+      <c r="I26" s="3">
+        <v>22</v>
+      </c>
       <c r="J26" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>110.583968</v>
       </c>
     </row>
     <row r="27" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="C27" s="2">
+        <v>10</v>
+      </c>
+      <c r="D27" s="2">
+        <v>59</v>
+      </c>
       <c r="E27" s="2">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>49</v>
+      </c>
+      <c r="F27" s="2">
+        <v>16</v>
+      </c>
+      <c r="G27" s="2">
+        <v>40</v>
+      </c>
+      <c r="H27" s="2">
+        <v>30</v>
+      </c>
+      <c r="I27" s="2">
+        <v>22</v>
       </c>
       <c r="J27" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>110.583968</v>
       </c>
     </row>
     <row r="28" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>5</v>
@@ -1150,7 +1381,7 @@
     </row>
     <row r="29" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>3</v>
@@ -1159,30 +1390,57 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="G29" s="3">
+        <v>27</v>
+      </c>
+      <c r="H29" s="3">
+        <v>30</v>
+      </c>
+      <c r="I29" s="3">
+        <v>17</v>
+      </c>
       <c r="J29" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>57.679592400000004</v>
       </c>
     </row>
     <row r="30" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="C30" s="2">
+        <v>11</v>
+      </c>
+      <c r="D30" s="2">
+        <v>123</v>
+      </c>
       <c r="E30" s="2">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>112</v>
+      </c>
+      <c r="F30" s="2">
+        <v>14</v>
+      </c>
+      <c r="G30" s="2">
+        <v>27</v>
+      </c>
+      <c r="H30" s="2">
+        <v>30</v>
+      </c>
+      <c r="I30" s="2">
+        <v>17</v>
       </c>
       <c r="J30" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>57.679592400000004</v>
       </c>
     </row>
     <row r="31" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>5</v>
@@ -1216,7 +1474,7 @@
     </row>
     <row r="32" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>3</v>
@@ -1225,30 +1483,57 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="G32" s="3">
+        <v>35</v>
+      </c>
+      <c r="H32" s="3">
+        <v>20</v>
+      </c>
+      <c r="I32" s="3">
+        <v>40</v>
+      </c>
       <c r="J32" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>117.28602666666664</v>
       </c>
     </row>
     <row r="33" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="C33" s="2">
+        <v>7</v>
+      </c>
+      <c r="D33" s="2">
+        <v>974</v>
+      </c>
       <c r="E33" s="2">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>967</v>
+      </c>
+      <c r="F33" s="2">
+        <v>17</v>
+      </c>
+      <c r="G33" s="2">
+        <v>35</v>
+      </c>
+      <c r="H33" s="2">
+        <v>20</v>
+      </c>
+      <c r="I33" s="2">
+        <v>40</v>
       </c>
       <c r="J33" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>117.28602666666664</v>
       </c>
     </row>
     <row r="34" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>5</v>
@@ -1282,7 +1567,7 @@
     </row>
     <row r="35" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>3</v>
@@ -1291,30 +1576,57 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="G35" s="3">
+        <v>20</v>
+      </c>
+      <c r="H35" s="3">
+        <v>15</v>
+      </c>
+      <c r="I35" s="3">
+        <v>20</v>
+      </c>
       <c r="J35" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>25.132719999999999</v>
       </c>
     </row>
     <row r="36" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="C36" s="2">
+        <v>3</v>
+      </c>
+      <c r="D36" s="2">
+        <v>643</v>
+      </c>
       <c r="E36" s="2">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>640</v>
+      </c>
+      <c r="F36" s="2">
+        <v>18</v>
+      </c>
+      <c r="G36" s="2">
+        <v>20</v>
+      </c>
+      <c r="H36" s="2">
+        <v>15</v>
+      </c>
+      <c r="I36" s="2">
+        <v>20</v>
       </c>
       <c r="J36" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>25.132719999999999</v>
       </c>
     </row>
     <row r="37" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>5</v>
@@ -1346,12 +1658,186 @@
         <v>25.132719999999999</v>
       </c>
     </row>
-    <row r="38" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="39" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="40" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="41" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="42" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="43" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="38" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E38" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G38" s="3">
+        <v>18</v>
+      </c>
+      <c r="H38" s="3">
+        <v>23</v>
+      </c>
+      <c r="I38" s="3">
+        <v>22</v>
+      </c>
+      <c r="J38" s="4">
+        <f t="shared" si="1"/>
+        <v>38.151468959999995</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" s="2">
+        <v>34</v>
+      </c>
+      <c r="D39" s="2">
+        <v>516</v>
+      </c>
+      <c r="E39" s="2">
+        <f t="shared" si="0"/>
+        <v>482</v>
+      </c>
+      <c r="F39" s="2">
+        <v>4</v>
+      </c>
+      <c r="G39" s="2">
+        <v>18</v>
+      </c>
+      <c r="H39" s="2">
+        <v>23</v>
+      </c>
+      <c r="I39" s="2">
+        <v>22</v>
+      </c>
+      <c r="J39" s="5">
+        <f t="shared" si="1"/>
+        <v>38.151468959999995</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C40" s="2">
+        <v>10</v>
+      </c>
+      <c r="D40" s="2">
+        <v>264</v>
+      </c>
+      <c r="E40" s="2">
+        <f t="shared" si="0"/>
+        <v>254</v>
+      </c>
+      <c r="F40" s="2">
+        <v>23</v>
+      </c>
+      <c r="G40" s="2">
+        <v>18</v>
+      </c>
+      <c r="H40" s="2">
+        <v>23</v>
+      </c>
+      <c r="I40" s="2">
+        <v>22</v>
+      </c>
+      <c r="J40" s="5">
+        <f t="shared" si="1"/>
+        <v>38.151468959999995</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E41" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G41" s="3">
+        <v>14</v>
+      </c>
+      <c r="H41" s="3">
+        <v>14</v>
+      </c>
+      <c r="I41" s="3">
+        <v>28</v>
+      </c>
+      <c r="J41" s="4">
+        <f t="shared" si="1"/>
+        <v>22.988061226666666</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E42" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F42" s="2">
+        <v>0</v>
+      </c>
+      <c r="G42" s="2">
+        <v>14</v>
+      </c>
+      <c r="H42" s="2">
+        <v>14</v>
+      </c>
+      <c r="I42" s="2">
+        <v>28</v>
+      </c>
+      <c r="J42" s="5">
+        <f t="shared" si="1"/>
+        <v>22.988061226666666</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C43" s="2">
+        <v>0</v>
+      </c>
+      <c r="D43" s="2">
+        <v>0</v>
+      </c>
+      <c r="E43" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F43" s="2">
+        <v>0</v>
+      </c>
+      <c r="G43" s="2">
+        <v>14</v>
+      </c>
+      <c r="H43" s="2">
+        <v>14</v>
+      </c>
+      <c r="I43" s="2">
+        <v>28</v>
+      </c>
+      <c r="J43" s="5">
+        <f t="shared" si="1"/>
+        <v>22.988061226666666</v>
+      </c>
+    </row>
     <row r="44" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="45" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="46" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2"/>

</xml_diff>